<commit_message>
Update AI Risk Assessment Calc
</commit_message>
<xml_diff>
--- a/AIGovernanceFramework/AI_Risk_Assessment_Calculator_v3.1.xlsx
+++ b/AIGovernanceFramework/AI_Risk_Assessment_Calculator_v3.1.xlsx
@@ -2,13 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corpdir-my.sharepoint.com/personal/rmirall_emea_corpdir_net/Documents/Documents/CODE/AIGovernanceFramework/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="11_B1FD3B786FB293D32CCE9F6121EF1EB916A17C9D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F27C40FE-9A28-4853-8813-041F308F0E20}"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F84D9234-F82C-4CA1-88A2-25C65A498709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1913,6 +1908,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2335,6 +2331,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4903,6 +4900,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5205,6 +5203,7 @@
     <mergeCell ref="B14:F14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7383,5 +7382,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>